<commit_message>
Release label print and GTIN workflow updates
</commit_message>
<xml_diff>
--- a/src/wb_marks_app/assets/gtin_request_template.xlsx
+++ b/src/wb_marks_app/assets/gtin_request_template.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9302"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="24195" windowHeight="14475"/>
@@ -11,23 +11,15 @@
     <sheet name="2. помощь" sheetId="4" r:id="rId2"/>
     <sheet name="catalogues" sheetId="2" state="hidden" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="144525"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <externalReferences>
+    <externalReference r:id="rId4"/>
+  </externalReferences>
+  <calcPr calcId="144525" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="580">
   <si>
     <t>СУБ-БРЕНД</t>
   </si>
@@ -1766,47 +1758,86 @@
 Наименование предприятия и префикс GCP:</t>
   </si>
   <si>
-    <t>ErLine</t>
+    <t>1</t>
+  </si>
+  <si>
+    <t>ОсОО "САДИЯН" 470009226</t>
+  </si>
+  <si>
+    <t>SAND Fashion</t>
+  </si>
+  <si>
+    <t>67030100</t>
+  </si>
+  <si>
+    <t>Арт.bnk_black, цвет: черный, р. 52</t>
   </si>
   <si>
     <t>Костюмы спортивные</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>ОсОО "ЭмирЛайн" (470905562)</t>
-  </si>
-  <si>
-    <t>Арт.cv_nk_white_smr, цвет: белый, р. 38</t>
-  </si>
-  <si>
-    <t>Арт.cv_nk_blue_smr, цвет: голубой, р. 38</t>
-  </si>
-  <si>
-    <t>Арт.cv_nk_blue_smr, цвет: голубой, р. 40</t>
-  </si>
-  <si>
-    <t>Арт.cv_nk_blue_smr, цвет: голубой, р. 42</t>
-  </si>
-  <si>
-    <t>Арт.cv_nk_blue_smr, цвет: голубой, р. 44</t>
-  </si>
-  <si>
-    <t>Арт.cv_nk_white_smr, цвет: белый, р. 44</t>
-  </si>
-  <si>
-    <t>Арт.cv_nk_white_smr, цвет: белый, р. 42</t>
-  </si>
-  <si>
-    <t>Арт.cv_nk_white_smr, цвет: белый, р. 40</t>
+    <t>Арт.bnk_black, цвет: черный, р. 50</t>
+  </si>
+  <si>
+    <t>Арт.bnk_black, цвет: черный, р. 54</t>
+  </si>
+  <si>
+    <t>Арт.bnk_black, цвет: черный, р. 48</t>
+  </si>
+  <si>
+    <t>Арт.bnk_black, цвет: черный, р. 46</t>
+  </si>
+  <si>
+    <t>Арт.bnk_hacks, цвет: хаки, р. 54</t>
+  </si>
+  <si>
+    <t>Арт.bnk_hacks, цвет: хаки, р. 52</t>
+  </si>
+  <si>
+    <t>Арт.bnk_hacks, цвет: хаки, р. 50</t>
+  </si>
+  <si>
+    <t>Арт.bnk_hacks, цвет: хаки, р. 48</t>
+  </si>
+  <si>
+    <t>Арт.bnk_hacks, цвет: хаки, р. 46</t>
+  </si>
+  <si>
+    <t>Арт.bnk_gray, цвет: серый, р. 46</t>
+  </si>
+  <si>
+    <t>Арт.bnk_gray, цвет: серый, р. 48</t>
+  </si>
+  <si>
+    <t>Арт.bnk_gray, цвет: серый, р. 50</t>
+  </si>
+  <si>
+    <t>Арт.bnk_gray, цвет: серый, р. 52</t>
+  </si>
+  <si>
+    <t>Арт.bnk_gray, цвет: серый, р. 54</t>
+  </si>
+  <si>
+    <t>Арт.bnk_blue, цвет: синий, р. 46</t>
+  </si>
+  <si>
+    <t>Арт.bnk_blue, цвет: синий, р. 48</t>
+  </si>
+  <si>
+    <t>Арт.bnk_blue, цвет: синий, р. 50</t>
+  </si>
+  <si>
+    <t>Арт.bnk_blue, цвет: синий, р. 52</t>
+  </si>
+  <si>
+    <t>Арт.bnk_blue, цвет: синий, р. 54</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1901,6 +1932,13 @@
       <charset val="204"/>
     </font>
     <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -1966,7 +2004,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
@@ -2002,7 +2040,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2020,17 +2062,31 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
   </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="1. данные_о_продукте"/>
+      <sheetName val="2. помощь"/>
+      <sheetName val="catalogues"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office 2013–2022">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2068,7 +2124,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
@@ -2174,7 +2230,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2316,7 +2372,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2324,70 +2380,70 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V36"/>
-  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
+  <dimension ref="A1:V134"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="45.1328125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="25.59765625" style="13" customWidth="1"/>
-    <col min="3" max="3" width="23.3984375" style="13" customWidth="1"/>
-    <col min="4" max="4" width="32.73046875" style="13" customWidth="1"/>
-    <col min="5" max="5" width="41.59765625" style="13" customWidth="1"/>
-    <col min="6" max="6" width="20.73046875" style="13" customWidth="1"/>
+    <col min="2" max="2" width="25.53125" style="13" customWidth="1"/>
+    <col min="3" max="3" width="23.46484375" style="13" customWidth="1"/>
+    <col min="4" max="4" width="32.6640625" style="13" customWidth="1"/>
+    <col min="5" max="5" width="41.53125" style="13" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" style="13" customWidth="1"/>
     <col min="7" max="7" width="24.86328125" style="13" customWidth="1"/>
     <col min="8" max="8" width="34" style="13" customWidth="1"/>
-    <col min="9" max="9" width="32.59765625" style="13" customWidth="1"/>
+    <col min="9" max="9" width="32.53125" style="13" customWidth="1"/>
     <col min="10" max="10" width="22.1328125" style="13" customWidth="1"/>
-    <col min="11" max="11" width="23.265625" style="13" customWidth="1"/>
+    <col min="11" max="11" width="23.33203125" style="13" customWidth="1"/>
     <col min="12" max="12" width="34.1328125" style="13" customWidth="1"/>
     <col min="13" max="13" width="29.86328125" style="13" customWidth="1"/>
-    <col min="14" max="14" width="25.73046875" style="13" customWidth="1"/>
-    <col min="15" max="15" width="22.73046875" style="13" customWidth="1"/>
+    <col min="14" max="14" width="25.6640625" style="13" customWidth="1"/>
+    <col min="15" max="15" width="22.6640625" style="13" customWidth="1"/>
     <col min="16" max="16" width="22.86328125" style="13" customWidth="1"/>
-    <col min="17" max="17" width="23.73046875" style="13" customWidth="1"/>
+    <col min="17" max="17" width="23.6640625" style="13" customWidth="1"/>
     <col min="18" max="18" width="51" style="13" customWidth="1"/>
     <col min="19" max="19" width="27" style="13" customWidth="1"/>
-    <col min="20" max="20" width="28.59765625" style="13" customWidth="1"/>
-    <col min="21" max="21" width="65.73046875" style="13" customWidth="1"/>
+    <col min="20" max="20" width="28.53125" style="13" customWidth="1"/>
+    <col min="21" max="21" width="65.6640625" style="13" customWidth="1"/>
     <col min="22" max="22" width="60" style="13" customWidth="1"/>
-    <col min="23" max="16384" width="9.1328125" style="3"/>
+    <col min="23" max="16384" width="9.06640625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="76.5" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="22" t="s">
         <v>553</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
-      <c r="S1" s="18"/>
-      <c r="T1" s="18"/>
-      <c r="U1" s="18"/>
-      <c r="V1" s="18"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
+      <c r="V1" s="22"/>
     </row>
     <row r="2" spans="1:22" ht="38.25" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="8" t="s">
         <v>554</v>
       </c>
-      <c r="B2" s="19" t="s">
-        <v>558</v>
-      </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
+      <c r="B2" s="23" t="s">
+        <v>556</v>
+      </c>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
       <c r="F2" s="9"/>
       <c r="G2" s="9"/>
       <c r="H2" s="9"/>
@@ -2613,17 +2669,17 @@
     <row r="6" spans="1:22" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.5"/>
     <row r="7" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A7" s="13" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B7" s="16"/>
       <c r="C7" s="16" t="s">
         <v>333</v>
       </c>
       <c r="D7" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E7" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
@@ -2641,11 +2697,11 @@
         <v>302</v>
       </c>
       <c r="Q7" s="16"/>
-      <c r="R7" s="17">
-        <v>10001359</v>
+      <c r="R7" s="17" t="s">
+        <v>558</v>
       </c>
       <c r="S7" s="16" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="T7" s="16" t="s">
         <v>111</v>
@@ -2659,17 +2715,17 @@
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A8" s="13" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B8" s="16"/>
       <c r="C8" s="16" t="s">
         <v>333</v>
       </c>
       <c r="D8" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E8" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
@@ -2687,11 +2743,11 @@
         <v>302</v>
       </c>
       <c r="Q8" s="16"/>
-      <c r="R8" s="17">
-        <v>10001359</v>
+      <c r="R8" s="17" t="s">
+        <v>558</v>
       </c>
       <c r="S8" s="16" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="T8" s="16" t="s">
         <v>111</v>
@@ -2705,17 +2761,17 @@
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A9" s="13" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B9" s="16"/>
       <c r="C9" s="16" t="s">
         <v>333</v>
       </c>
       <c r="D9" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E9" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
@@ -2733,11 +2789,11 @@
         <v>302</v>
       </c>
       <c r="Q9" s="16"/>
-      <c r="R9" s="17">
-        <v>10001359</v>
+      <c r="R9" s="17" t="s">
+        <v>558</v>
       </c>
       <c r="S9" s="16" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="T9" s="16" t="s">
         <v>111</v>
@@ -2751,17 +2807,17 @@
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A10" s="13" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B10" s="16"/>
       <c r="C10" s="16" t="s">
         <v>333</v>
       </c>
       <c r="D10" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E10" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
@@ -2779,11 +2835,11 @@
         <v>302</v>
       </c>
       <c r="Q10" s="16"/>
-      <c r="R10" s="17">
-        <v>10001359</v>
+      <c r="R10" s="17" t="s">
+        <v>558</v>
       </c>
       <c r="S10" s="16" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="T10" s="16" t="s">
         <v>111</v>
@@ -2797,17 +2853,17 @@
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A11" s="13" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="16" t="s">
         <v>333</v>
       </c>
       <c r="D11" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E11" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
@@ -2825,11 +2881,11 @@
         <v>302</v>
       </c>
       <c r="Q11" s="16"/>
-      <c r="R11" s="17">
-        <v>10001359</v>
+      <c r="R11" s="17" t="s">
+        <v>558</v>
       </c>
       <c r="S11" s="16" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="T11" s="16" t="s">
         <v>111</v>
@@ -2843,17 +2899,17 @@
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A12" s="13" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B12" s="16"/>
       <c r="C12" s="16" t="s">
         <v>333</v>
       </c>
       <c r="D12" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E12" t="s">
-        <v>561</v>
+        <v>569</v>
       </c>
       <c r="F12" s="16"/>
       <c r="G12" s="16"/>
@@ -2871,11 +2927,11 @@
         <v>302</v>
       </c>
       <c r="Q12" s="16"/>
-      <c r="R12" s="17">
-        <v>10001359</v>
+      <c r="R12" s="17" t="s">
+        <v>558</v>
       </c>
       <c r="S12" s="16" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="T12" s="16" t="s">
         <v>111</v>
@@ -2889,17 +2945,17 @@
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A13" s="13" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16" t="s">
         <v>333</v>
       </c>
       <c r="D13" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E13" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
@@ -2917,11 +2973,11 @@
         <v>302</v>
       </c>
       <c r="Q13" s="16"/>
-      <c r="R13" s="17">
-        <v>10001359</v>
+      <c r="R13" s="17" t="s">
+        <v>558</v>
       </c>
       <c r="S13" s="16" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="T13" s="16" t="s">
         <v>111</v>
@@ -2935,17 +2991,17 @@
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.5">
       <c r="A14" s="13" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="16" t="s">
         <v>333</v>
       </c>
       <c r="D14" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E14" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
@@ -2963,11 +3019,11 @@
         <v>302</v>
       </c>
       <c r="Q14" s="16"/>
-      <c r="R14" s="17">
-        <v>10001359</v>
+      <c r="R14" s="17" t="s">
+        <v>558</v>
       </c>
       <c r="S14" s="16" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="T14" s="16" t="s">
         <v>111</v>
@@ -2980,370 +3036,2025 @@
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.5">
-      <c r="C15" s="16"/>
-      <c r="D15"/>
-      <c r="E15"/>
-      <c r="O15" s="16"/>
-      <c r="P15" s="16"/>
-      <c r="R15" s="17"/>
-      <c r="S15" s="16"/>
-      <c r="T15" s="16"/>
-      <c r="U15" s="16"/>
-      <c r="V15" s="16"/>
+      <c r="A15" s="13" t="s">
+        <v>557</v>
+      </c>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="D15" t="s">
+        <v>560</v>
+      </c>
+      <c r="E15" t="s">
+        <v>566</v>
+      </c>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="16"/>
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="P15" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q15" s="16"/>
+      <c r="R15" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="S15" s="16" t="s">
+        <v>555</v>
+      </c>
+      <c r="T15" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="U15" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="V15" s="16" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.5">
-      <c r="C16" s="16"/>
-      <c r="D16"/>
-      <c r="E16"/>
-      <c r="O16" s="16"/>
-      <c r="P16" s="16"/>
-      <c r="R16" s="17"/>
-      <c r="S16" s="16"/>
-      <c r="T16" s="16"/>
-      <c r="U16" s="16"/>
-      <c r="V16" s="16"/>
-    </row>
-    <row r="17" spans="2:22" x14ac:dyDescent="0.5">
-      <c r="C17" s="16"/>
-      <c r="D17"/>
-      <c r="E17"/>
-      <c r="O17" s="16"/>
-      <c r="P17" s="16"/>
-      <c r="R17" s="17"/>
-      <c r="S17" s="16"/>
-      <c r="T17" s="16"/>
-      <c r="U17" s="16"/>
-      <c r="V17" s="16"/>
-    </row>
-    <row r="18" spans="2:22" x14ac:dyDescent="0.5">
-      <c r="C18" s="16"/>
-      <c r="D18"/>
-      <c r="E18"/>
-      <c r="O18" s="16"/>
-      <c r="P18" s="16"/>
-      <c r="R18" s="17"/>
-      <c r="S18" s="16"/>
-      <c r="T18" s="16"/>
-      <c r="U18" s="16"/>
-      <c r="V18" s="16"/>
-    </row>
-    <row r="19" spans="2:22" x14ac:dyDescent="0.5">
-      <c r="C19" s="16"/>
-      <c r="D19"/>
-      <c r="E19"/>
-      <c r="O19" s="16"/>
-      <c r="P19" s="16"/>
-      <c r="R19" s="17"/>
-      <c r="S19" s="16"/>
-      <c r="T19" s="16"/>
-      <c r="U19" s="16"/>
-      <c r="V19" s="16"/>
-    </row>
-    <row r="20" spans="2:22" x14ac:dyDescent="0.5">
-      <c r="C20" s="16"/>
-      <c r="D20"/>
-      <c r="E20"/>
-      <c r="O20" s="16"/>
-      <c r="P20" s="16"/>
-      <c r="R20" s="17"/>
-      <c r="S20" s="16"/>
-      <c r="T20" s="16"/>
-      <c r="U20" s="16"/>
-      <c r="V20" s="16"/>
-    </row>
-    <row r="21" spans="2:22" x14ac:dyDescent="0.5">
-      <c r="C21" s="16"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="O21" s="16"/>
-      <c r="P21" s="16"/>
-      <c r="R21" s="17"/>
-      <c r="S21" s="16"/>
-      <c r="T21" s="16"/>
-      <c r="U21" s="16"/>
-      <c r="V21" s="16"/>
-    </row>
-    <row r="22" spans="2:22" x14ac:dyDescent="0.5">
-      <c r="B22" s="16"/>
-      <c r="C22" s="16"/>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="F22" s="16"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="16"/>
-      <c r="O22" s="16"/>
-      <c r="P22" s="16"/>
-      <c r="Q22" s="16"/>
-      <c r="R22" s="17"/>
-      <c r="S22" s="16"/>
-      <c r="T22" s="16"/>
-      <c r="U22" s="16"/>
-      <c r="V22" s="16"/>
-    </row>
-    <row r="23" spans="2:22" x14ac:dyDescent="0.5">
-      <c r="B23" s="16"/>
-      <c r="C23" s="16"/>
-      <c r="D23"/>
-      <c r="E23"/>
-      <c r="F23" s="16"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="16"/>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="16"/>
-      <c r="O23" s="16"/>
-      <c r="P23" s="16"/>
-      <c r="Q23" s="16"/>
-      <c r="R23" s="17"/>
-      <c r="S23" s="16"/>
-      <c r="T23" s="16"/>
-      <c r="U23" s="16"/>
-      <c r="V23" s="16"/>
-    </row>
-    <row r="24" spans="2:22" x14ac:dyDescent="0.5">
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24"/>
-      <c r="E24"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="16"/>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="16"/>
-      <c r="O24" s="16"/>
-      <c r="P24" s="16"/>
-      <c r="Q24" s="16"/>
-      <c r="R24" s="17"/>
-      <c r="S24" s="16"/>
-      <c r="T24" s="16"/>
-      <c r="U24" s="16"/>
-      <c r="V24" s="16"/>
-    </row>
-    <row r="25" spans="2:22" x14ac:dyDescent="0.5">
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25"/>
-      <c r="E25"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="16"/>
-      <c r="O25" s="16"/>
-      <c r="P25" s="16"/>
-      <c r="Q25" s="16"/>
-      <c r="R25" s="17"/>
-      <c r="S25" s="16"/>
-      <c r="T25" s="16"/>
-      <c r="U25" s="16"/>
-      <c r="V25" s="16"/>
-    </row>
-    <row r="26" spans="2:22" x14ac:dyDescent="0.5">
-      <c r="C26" s="16"/>
-      <c r="D26"/>
-      <c r="E26"/>
-      <c r="O26" s="16"/>
-      <c r="P26" s="16"/>
-      <c r="R26" s="17"/>
-      <c r="S26" s="16"/>
-      <c r="T26" s="16"/>
-      <c r="U26" s="16"/>
-      <c r="V26" s="16"/>
-    </row>
-    <row r="27" spans="2:22" x14ac:dyDescent="0.5">
+      <c r="A16" s="13" t="s">
+        <v>557</v>
+      </c>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="D16" t="s">
+        <v>560</v>
+      </c>
+      <c r="E16" t="s">
+        <v>565</v>
+      </c>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="P16" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="S16" s="16" t="s">
+        <v>555</v>
+      </c>
+      <c r="T16" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="U16" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="V16" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A17" s="13" t="s">
+        <v>557</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="D17" t="s">
+        <v>560</v>
+      </c>
+      <c r="E17" t="s">
+        <v>570</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="16"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="P17" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q17" s="16"/>
+      <c r="R17" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="S17" s="16" t="s">
+        <v>555</v>
+      </c>
+      <c r="T17" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="U17" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="V17" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A18" s="13" t="s">
+        <v>557</v>
+      </c>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="D18" t="s">
+        <v>560</v>
+      </c>
+      <c r="E18" t="s">
+        <v>571</v>
+      </c>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="P18" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="S18" s="16" t="s">
+        <v>555</v>
+      </c>
+      <c r="T18" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="U18" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="V18" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A19" s="13" t="s">
+        <v>557</v>
+      </c>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="D19" t="s">
+        <v>560</v>
+      </c>
+      <c r="E19" t="s">
+        <v>572</v>
+      </c>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="16"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="16"/>
+      <c r="L19" s="16"/>
+      <c r="M19" s="16"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="P19" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q19" s="16"/>
+      <c r="R19" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="S19" s="16" t="s">
+        <v>555</v>
+      </c>
+      <c r="T19" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="U19" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="V19" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A20" s="13" t="s">
+        <v>557</v>
+      </c>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="D20" t="s">
+        <v>560</v>
+      </c>
+      <c r="E20" t="s">
+        <v>573</v>
+      </c>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="P20" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q20" s="16"/>
+      <c r="R20" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="S20" s="16" t="s">
+        <v>555</v>
+      </c>
+      <c r="T20" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="U20" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="V20" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A21" s="13" t="s">
+        <v>557</v>
+      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16" t="s">
+        <v>333</v>
+      </c>
+      <c r="D21" t="s">
+        <v>560</v>
+      </c>
+      <c r="E21" t="s">
+        <v>574</v>
+      </c>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="16"/>
+      <c r="O21" s="16" t="s">
+        <v>425</v>
+      </c>
+      <c r="P21" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q21" s="16"/>
+      <c r="R21" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="S21" s="16" t="s">
+        <v>555</v>
+      </c>
+      <c r="T21" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="U21" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="V21" s="16" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A22" s="19" t="s">
+        <v>557</v>
+      </c>
+      <c r="B22" s="20"/>
+      <c r="C22" s="20" t="s">
+        <v>333</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>560</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>575</v>
+      </c>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="20"/>
+      <c r="M22" s="20"/>
+      <c r="N22" s="20"/>
+      <c r="O22" s="20" t="s">
+        <v>425</v>
+      </c>
+      <c r="P22" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q22" s="20"/>
+      <c r="R22" s="21" t="s">
+        <v>558</v>
+      </c>
+      <c r="S22" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="T22" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="U22" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="V22" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A23" s="19" t="s">
+        <v>557</v>
+      </c>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20" t="s">
+        <v>333</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>560</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>576</v>
+      </c>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
+      <c r="L23" s="20"/>
+      <c r="M23" s="20"/>
+      <c r="N23" s="20"/>
+      <c r="O23" s="20" t="s">
+        <v>425</v>
+      </c>
+      <c r="P23" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q23" s="20"/>
+      <c r="R23" s="21" t="s">
+        <v>558</v>
+      </c>
+      <c r="S23" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="T23" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="U23" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="V23" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A24" s="19" t="s">
+        <v>557</v>
+      </c>
+      <c r="B24" s="20"/>
+      <c r="C24" s="20" t="s">
+        <v>333</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>560</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>577</v>
+      </c>
+      <c r="F24" s="20"/>
+      <c r="G24" s="20"/>
+      <c r="H24" s="20"/>
+      <c r="I24" s="20"/>
+      <c r="J24" s="20"/>
+      <c r="K24" s="20"/>
+      <c r="L24" s="20"/>
+      <c r="M24" s="20"/>
+      <c r="N24" s="20"/>
+      <c r="O24" s="20" t="s">
+        <v>425</v>
+      </c>
+      <c r="P24" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q24" s="20"/>
+      <c r="R24" s="21" t="s">
+        <v>558</v>
+      </c>
+      <c r="S24" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="T24" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="U24" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="V24" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A25" s="19" t="s">
+        <v>557</v>
+      </c>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20" t="s">
+        <v>333</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>560</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>578</v>
+      </c>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="20"/>
+      <c r="K25" s="20"/>
+      <c r="L25" s="20"/>
+      <c r="M25" s="20"/>
+      <c r="N25" s="20"/>
+      <c r="O25" s="20" t="s">
+        <v>425</v>
+      </c>
+      <c r="P25" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q25" s="20"/>
+      <c r="R25" s="21" t="s">
+        <v>558</v>
+      </c>
+      <c r="S25" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="T25" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="U25" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="V25" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A26" s="19" t="s">
+        <v>557</v>
+      </c>
+      <c r="B26" s="20"/>
+      <c r="C26" s="20" t="s">
+        <v>333</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>560</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>579</v>
+      </c>
+      <c r="F26" s="20"/>
+      <c r="G26" s="20"/>
+      <c r="H26" s="20"/>
+      <c r="I26" s="20"/>
+      <c r="J26" s="20"/>
+      <c r="K26" s="20"/>
+      <c r="L26" s="20"/>
+      <c r="M26" s="20"/>
+      <c r="N26" s="20"/>
+      <c r="O26" s="20" t="s">
+        <v>425</v>
+      </c>
+      <c r="P26" s="20" t="s">
+        <v>302</v>
+      </c>
+      <c r="Q26" s="20"/>
+      <c r="R26" s="21" t="s">
+        <v>558</v>
+      </c>
+      <c r="S26" s="20" t="s">
+        <v>555</v>
+      </c>
+      <c r="T26" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="U26" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="V26" s="20" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A27" s="16"/>
       <c r="C27" s="16"/>
-      <c r="D27"/>
-      <c r="E27"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
       <c r="O27" s="16"/>
       <c r="P27" s="16"/>
-      <c r="R27" s="17"/>
+      <c r="R27" s="16"/>
       <c r="S27" s="16"/>
       <c r="T27" s="16"/>
       <c r="U27" s="16"/>
       <c r="V27" s="16"/>
     </row>
-    <row r="28" spans="2:22" x14ac:dyDescent="0.5">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A28" s="16"/>
       <c r="C28" s="16"/>
-      <c r="D28"/>
-      <c r="E28"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
       <c r="O28" s="16"/>
       <c r="P28" s="16"/>
-      <c r="R28" s="17"/>
+      <c r="R28" s="16"/>
       <c r="S28" s="16"/>
       <c r="T28" s="16"/>
       <c r="U28" s="16"/>
       <c r="V28" s="16"/>
     </row>
-    <row r="29" spans="2:22" x14ac:dyDescent="0.5">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A29" s="16"/>
       <c r="C29" s="16"/>
-      <c r="D29"/>
-      <c r="E29"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
       <c r="O29" s="16"/>
       <c r="P29" s="16"/>
-      <c r="R29" s="17"/>
+      <c r="R29" s="16"/>
       <c r="S29" s="16"/>
       <c r="T29" s="16"/>
       <c r="U29" s="16"/>
       <c r="V29" s="16"/>
     </row>
-    <row r="30" spans="2:22" x14ac:dyDescent="0.5">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A30" s="16"/>
       <c r="C30" s="16"/>
-      <c r="D30"/>
-      <c r="E30"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
       <c r="O30" s="16"/>
       <c r="P30" s="16"/>
-      <c r="R30" s="17"/>
+      <c r="R30" s="16"/>
       <c r="S30" s="16"/>
       <c r="T30" s="16"/>
       <c r="U30" s="16"/>
       <c r="V30" s="16"/>
     </row>
-    <row r="31" spans="2:22" x14ac:dyDescent="0.5">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A31" s="16"/>
       <c r="C31" s="16"/>
-      <c r="D31"/>
-      <c r="E31"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
       <c r="O31" s="16"/>
       <c r="P31" s="16"/>
-      <c r="R31" s="17"/>
+      <c r="R31" s="16"/>
       <c r="S31" s="16"/>
       <c r="T31" s="16"/>
       <c r="U31" s="16"/>
       <c r="V31" s="16"/>
     </row>
-    <row r="32" spans="2:22" x14ac:dyDescent="0.5">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A32" s="16"/>
       <c r="C32" s="16"/>
-      <c r="D32"/>
-      <c r="E32"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
       <c r="O32" s="16"/>
       <c r="P32" s="16"/>
-      <c r="R32" s="17"/>
+      <c r="R32" s="16"/>
       <c r="S32" s="16"/>
       <c r="T32" s="16"/>
       <c r="U32" s="16"/>
       <c r="V32" s="16"/>
     </row>
-    <row r="33" spans="3:22" x14ac:dyDescent="0.5">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A33" s="16"/>
       <c r="C33" s="16"/>
-      <c r="D33"/>
-      <c r="E33"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
       <c r="O33" s="16"/>
       <c r="P33" s="16"/>
-      <c r="R33" s="17"/>
+      <c r="R33" s="16"/>
       <c r="S33" s="16"/>
       <c r="T33" s="16"/>
       <c r="U33" s="16"/>
       <c r="V33" s="16"/>
     </row>
-    <row r="34" spans="3:22" x14ac:dyDescent="0.5">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A34" s="16"/>
       <c r="C34" s="16"/>
-      <c r="D34"/>
-      <c r="E34"/>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
       <c r="O34" s="16"/>
       <c r="P34" s="16"/>
-      <c r="R34" s="17"/>
+      <c r="R34" s="16"/>
       <c r="S34" s="16"/>
       <c r="T34" s="16"/>
       <c r="U34" s="16"/>
       <c r="V34" s="16"/>
     </row>
-    <row r="35" spans="3:22" x14ac:dyDescent="0.5">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A35" s="16"/>
       <c r="C35" s="16"/>
-      <c r="D35"/>
-      <c r="E35"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
       <c r="O35" s="16"/>
       <c r="P35" s="16"/>
-      <c r="R35" s="17"/>
+      <c r="R35" s="16"/>
       <c r="S35" s="16"/>
       <c r="T35" s="16"/>
       <c r="U35" s="16"/>
       <c r="V35" s="16"/>
     </row>
-    <row r="36" spans="3:22" x14ac:dyDescent="0.5">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A36" s="16"/>
       <c r="C36" s="16"/>
-      <c r="D36"/>
-      <c r="E36"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
       <c r="O36" s="16"/>
       <c r="P36" s="16"/>
-      <c r="R36" s="17"/>
+      <c r="R36" s="16"/>
       <c r="S36" s="16"/>
       <c r="T36" s="16"/>
       <c r="U36" s="16"/>
       <c r="V36" s="16"/>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A37" s="16"/>
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="O37" s="16"/>
+      <c r="P37" s="16"/>
+      <c r="R37" s="16"/>
+      <c r="S37" s="16"/>
+      <c r="T37" s="16"/>
+      <c r="U37" s="16"/>
+      <c r="V37" s="16"/>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="O38" s="16"/>
+      <c r="P38" s="16"/>
+      <c r="R38" s="16"/>
+      <c r="S38" s="16"/>
+      <c r="T38" s="16"/>
+      <c r="U38" s="16"/>
+      <c r="V38" s="16"/>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="16"/>
+      <c r="E39" s="16"/>
+      <c r="O39" s="16"/>
+      <c r="P39" s="16"/>
+      <c r="R39" s="16"/>
+      <c r="S39" s="16"/>
+      <c r="T39" s="16"/>
+      <c r="U39" s="16"/>
+      <c r="V39" s="16"/>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A40" s="16"/>
+      <c r="C40" s="16"/>
+      <c r="D40" s="16"/>
+      <c r="E40" s="16"/>
+      <c r="O40" s="16"/>
+      <c r="P40" s="16"/>
+      <c r="R40" s="16"/>
+      <c r="S40" s="16"/>
+      <c r="T40" s="16"/>
+      <c r="U40" s="16"/>
+      <c r="V40" s="16"/>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A41" s="16"/>
+      <c r="C41" s="16"/>
+      <c r="D41" s="16"/>
+      <c r="E41" s="16"/>
+      <c r="O41" s="16"/>
+      <c r="P41" s="16"/>
+      <c r="R41" s="16"/>
+      <c r="S41" s="16"/>
+      <c r="T41" s="16"/>
+      <c r="U41" s="16"/>
+      <c r="V41" s="16"/>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A42" s="16"/>
+      <c r="C42" s="16"/>
+      <c r="D42" s="16"/>
+      <c r="E42" s="16"/>
+      <c r="O42" s="16"/>
+      <c r="P42" s="16"/>
+      <c r="R42" s="16"/>
+      <c r="S42" s="16"/>
+      <c r="T42" s="16"/>
+      <c r="U42" s="16"/>
+      <c r="V42" s="16"/>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A43" s="16"/>
+      <c r="C43" s="16"/>
+      <c r="D43" s="16"/>
+      <c r="E43" s="16"/>
+      <c r="O43" s="16"/>
+      <c r="P43" s="16"/>
+      <c r="R43" s="16"/>
+      <c r="S43" s="16"/>
+      <c r="T43" s="16"/>
+      <c r="U43" s="16"/>
+      <c r="V43" s="16"/>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A44" s="16"/>
+      <c r="C44" s="16"/>
+      <c r="D44" s="16"/>
+      <c r="E44" s="16"/>
+      <c r="O44" s="16"/>
+      <c r="P44" s="16"/>
+      <c r="R44" s="16"/>
+      <c r="S44" s="16"/>
+      <c r="T44" s="16"/>
+      <c r="U44" s="16"/>
+      <c r="V44" s="16"/>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A45" s="16"/>
+      <c r="C45" s="16"/>
+      <c r="D45" s="16"/>
+      <c r="E45" s="16"/>
+      <c r="O45" s="16"/>
+      <c r="P45" s="16"/>
+      <c r="R45" s="16"/>
+      <c r="S45" s="16"/>
+      <c r="T45" s="16"/>
+      <c r="U45" s="16"/>
+      <c r="V45" s="16"/>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A46" s="16"/>
+      <c r="C46" s="16"/>
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
+      <c r="O46" s="16"/>
+      <c r="P46" s="16"/>
+      <c r="R46" s="16"/>
+      <c r="S46" s="16"/>
+      <c r="T46" s="16"/>
+      <c r="U46" s="16"/>
+      <c r="V46" s="16"/>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A47" s="16"/>
+      <c r="C47" s="16"/>
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+      <c r="O47" s="16"/>
+      <c r="P47" s="16"/>
+      <c r="R47" s="16"/>
+      <c r="S47" s="16"/>
+      <c r="T47" s="16"/>
+      <c r="U47" s="16"/>
+      <c r="V47" s="16"/>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A48" s="16"/>
+      <c r="C48" s="16"/>
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
+      <c r="O48" s="16"/>
+      <c r="P48" s="16"/>
+      <c r="R48" s="16"/>
+      <c r="S48" s="16"/>
+      <c r="T48" s="16"/>
+      <c r="U48" s="16"/>
+      <c r="V48" s="16"/>
+    </row>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A49" s="16"/>
+      <c r="C49" s="16"/>
+      <c r="D49" s="16"/>
+      <c r="E49" s="16"/>
+      <c r="O49" s="16"/>
+      <c r="P49" s="16"/>
+      <c r="R49" s="16"/>
+      <c r="S49" s="16"/>
+      <c r="T49" s="16"/>
+      <c r="U49" s="16"/>
+      <c r="V49" s="16"/>
+    </row>
+    <row r="50" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A50" s="16"/>
+      <c r="C50" s="16"/>
+      <c r="D50" s="16"/>
+      <c r="E50" s="16"/>
+      <c r="O50" s="16"/>
+      <c r="P50" s="16"/>
+      <c r="R50" s="16"/>
+      <c r="S50" s="16"/>
+      <c r="T50" s="16"/>
+      <c r="U50" s="16"/>
+      <c r="V50" s="16"/>
+    </row>
+    <row r="51" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A51" s="16"/>
+      <c r="C51" s="16"/>
+      <c r="D51" s="16"/>
+      <c r="E51" s="16"/>
+      <c r="O51" s="16"/>
+      <c r="P51" s="16"/>
+      <c r="R51" s="16"/>
+      <c r="S51" s="16"/>
+      <c r="T51" s="16"/>
+      <c r="U51" s="16"/>
+      <c r="V51" s="16"/>
+    </row>
+    <row r="52" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A52" s="16"/>
+      <c r="C52" s="16"/>
+      <c r="D52" s="16"/>
+      <c r="E52" s="16"/>
+      <c r="O52" s="16"/>
+      <c r="P52" s="16"/>
+      <c r="R52" s="16"/>
+      <c r="S52" s="16"/>
+      <c r="T52" s="16"/>
+      <c r="U52" s="16"/>
+      <c r="V52" s="16"/>
+    </row>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A53" s="16"/>
+      <c r="C53" s="16"/>
+      <c r="D53" s="16"/>
+      <c r="E53" s="16"/>
+      <c r="O53" s="16"/>
+      <c r="P53" s="16"/>
+      <c r="R53" s="16"/>
+      <c r="S53" s="16"/>
+      <c r="T53" s="16"/>
+      <c r="U53" s="16"/>
+      <c r="V53" s="16"/>
+    </row>
+    <row r="54" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A54" s="16"/>
+      <c r="C54" s="16"/>
+      <c r="D54" s="16"/>
+      <c r="E54" s="16"/>
+      <c r="O54" s="16"/>
+      <c r="P54" s="16"/>
+      <c r="R54" s="16"/>
+      <c r="S54" s="16"/>
+      <c r="T54" s="16"/>
+      <c r="U54" s="16"/>
+      <c r="V54" s="16"/>
+    </row>
+    <row r="55" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A55" s="16"/>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
+      <c r="O55" s="16"/>
+      <c r="P55" s="16"/>
+      <c r="R55" s="16"/>
+      <c r="S55" s="16"/>
+      <c r="T55" s="16"/>
+      <c r="U55" s="16"/>
+      <c r="V55" s="16"/>
+    </row>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A56" s="16"/>
+      <c r="C56" s="16"/>
+      <c r="D56" s="16"/>
+      <c r="E56" s="16"/>
+      <c r="O56" s="16"/>
+      <c r="P56" s="16"/>
+      <c r="R56" s="16"/>
+      <c r="S56" s="16"/>
+      <c r="T56" s="16"/>
+      <c r="U56" s="16"/>
+      <c r="V56" s="16"/>
+    </row>
+    <row r="57" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A57" s="16"/>
+      <c r="C57" s="16"/>
+      <c r="D57" s="16"/>
+      <c r="E57" s="16"/>
+      <c r="O57" s="16"/>
+      <c r="P57" s="16"/>
+      <c r="R57" s="16"/>
+      <c r="S57" s="16"/>
+      <c r="T57" s="16"/>
+      <c r="U57" s="16"/>
+      <c r="V57" s="16"/>
+    </row>
+    <row r="58" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A58" s="16"/>
+      <c r="C58" s="16"/>
+      <c r="D58" s="16"/>
+      <c r="E58" s="16"/>
+      <c r="O58" s="16"/>
+      <c r="P58" s="16"/>
+      <c r="R58" s="16"/>
+      <c r="S58" s="16"/>
+      <c r="T58" s="16"/>
+      <c r="U58" s="16"/>
+      <c r="V58" s="16"/>
+    </row>
+    <row r="59" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A59" s="16"/>
+      <c r="C59" s="16"/>
+      <c r="D59" s="16"/>
+      <c r="E59" s="16"/>
+      <c r="O59" s="16"/>
+      <c r="P59" s="16"/>
+      <c r="R59" s="16"/>
+      <c r="S59" s="16"/>
+      <c r="T59" s="16"/>
+      <c r="U59" s="16"/>
+      <c r="V59" s="16"/>
+    </row>
+    <row r="60" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A60" s="16"/>
+      <c r="C60" s="16"/>
+      <c r="D60" s="16"/>
+      <c r="E60" s="16"/>
+      <c r="O60" s="16"/>
+      <c r="P60" s="16"/>
+      <c r="R60" s="16"/>
+      <c r="S60" s="16"/>
+      <c r="T60" s="16"/>
+      <c r="U60" s="16"/>
+      <c r="V60" s="16"/>
+    </row>
+    <row r="61" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A61" s="16"/>
+      <c r="C61" s="16"/>
+      <c r="D61" s="16"/>
+      <c r="E61" s="16"/>
+      <c r="O61" s="16"/>
+      <c r="P61" s="16"/>
+      <c r="R61" s="16"/>
+      <c r="S61" s="16"/>
+      <c r="T61" s="16"/>
+      <c r="U61" s="16"/>
+      <c r="V61" s="16"/>
+    </row>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A62" s="16"/>
+      <c r="C62" s="16"/>
+      <c r="D62" s="16"/>
+      <c r="E62" s="16"/>
+      <c r="O62" s="16"/>
+      <c r="P62" s="16"/>
+      <c r="R62" s="16"/>
+      <c r="S62" s="16"/>
+      <c r="T62" s="16"/>
+      <c r="U62" s="16"/>
+      <c r="V62" s="16"/>
+    </row>
+    <row r="63" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A63" s="16"/>
+      <c r="C63" s="16"/>
+      <c r="D63" s="16"/>
+      <c r="E63" s="16"/>
+      <c r="O63" s="16"/>
+      <c r="P63" s="16"/>
+      <c r="R63" s="16"/>
+      <c r="S63" s="16"/>
+      <c r="T63" s="16"/>
+      <c r="U63" s="16"/>
+      <c r="V63" s="16"/>
+    </row>
+    <row r="64" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A64" s="16"/>
+      <c r="C64" s="16"/>
+      <c r="D64" s="16"/>
+      <c r="E64" s="16"/>
+      <c r="O64" s="16"/>
+      <c r="P64" s="16"/>
+      <c r="R64" s="16"/>
+      <c r="S64" s="16"/>
+      <c r="T64" s="16"/>
+      <c r="U64" s="16"/>
+      <c r="V64" s="16"/>
+    </row>
+    <row r="65" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A65" s="16"/>
+      <c r="C65" s="16"/>
+      <c r="D65" s="16"/>
+      <c r="E65" s="16"/>
+      <c r="O65" s="16"/>
+      <c r="P65" s="16"/>
+      <c r="R65" s="16"/>
+      <c r="S65" s="16"/>
+      <c r="T65" s="16"/>
+      <c r="U65" s="16"/>
+      <c r="V65" s="16"/>
+    </row>
+    <row r="66" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A66" s="16"/>
+      <c r="C66" s="16"/>
+      <c r="D66" s="16"/>
+      <c r="E66" s="16"/>
+      <c r="O66" s="16"/>
+      <c r="P66" s="16"/>
+      <c r="R66" s="16"/>
+      <c r="S66" s="16"/>
+      <c r="T66" s="16"/>
+      <c r="U66" s="16"/>
+      <c r="V66" s="16"/>
+    </row>
+    <row r="67" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A67" s="16"/>
+      <c r="C67" s="16"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="O67" s="16"/>
+      <c r="P67" s="16"/>
+      <c r="R67" s="16"/>
+      <c r="S67" s="16"/>
+      <c r="T67" s="16"/>
+      <c r="U67" s="16"/>
+      <c r="V67" s="16"/>
+    </row>
+    <row r="68" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A68" s="16"/>
+      <c r="C68" s="16"/>
+      <c r="D68" s="16"/>
+      <c r="E68" s="16"/>
+      <c r="O68" s="16"/>
+      <c r="P68" s="16"/>
+      <c r="R68" s="16"/>
+      <c r="S68" s="16"/>
+      <c r="T68" s="16"/>
+      <c r="U68" s="16"/>
+      <c r="V68" s="16"/>
+    </row>
+    <row r="69" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A69" s="16"/>
+      <c r="C69" s="16"/>
+      <c r="D69" s="16"/>
+      <c r="E69" s="16"/>
+      <c r="O69" s="16"/>
+      <c r="P69" s="16"/>
+      <c r="R69" s="16"/>
+      <c r="S69" s="16"/>
+      <c r="T69" s="16"/>
+      <c r="U69" s="16"/>
+      <c r="V69" s="16"/>
+    </row>
+    <row r="70" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A70" s="16"/>
+      <c r="C70" s="16"/>
+      <c r="D70" s="16"/>
+      <c r="E70" s="16"/>
+      <c r="O70" s="16"/>
+      <c r="P70" s="16"/>
+      <c r="R70" s="16"/>
+      <c r="S70" s="16"/>
+      <c r="T70" s="16"/>
+      <c r="U70" s="16"/>
+      <c r="V70" s="16"/>
+    </row>
+    <row r="71" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A71" s="16"/>
+      <c r="C71" s="16"/>
+      <c r="D71" s="16"/>
+      <c r="E71" s="16"/>
+      <c r="O71" s="16"/>
+      <c r="P71" s="16"/>
+      <c r="R71" s="16"/>
+      <c r="S71" s="16"/>
+      <c r="T71" s="16"/>
+      <c r="U71" s="16"/>
+      <c r="V71" s="16"/>
+    </row>
+    <row r="72" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A72" s="16"/>
+      <c r="C72" s="16"/>
+      <c r="D72" s="16"/>
+      <c r="E72" s="16"/>
+      <c r="O72" s="16"/>
+      <c r="P72" s="16"/>
+      <c r="R72" s="16"/>
+      <c r="S72" s="16"/>
+      <c r="T72" s="16"/>
+      <c r="U72" s="16"/>
+      <c r="V72" s="16"/>
+    </row>
+    <row r="73" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A73" s="16"/>
+      <c r="C73" s="16"/>
+      <c r="D73" s="16"/>
+      <c r="E73" s="16"/>
+      <c r="O73" s="16"/>
+      <c r="P73" s="16"/>
+      <c r="R73" s="16"/>
+      <c r="S73" s="16"/>
+      <c r="T73" s="16"/>
+      <c r="U73" s="16"/>
+      <c r="V73" s="16"/>
+    </row>
+    <row r="74" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A74" s="16"/>
+      <c r="C74" s="16"/>
+      <c r="D74" s="16"/>
+      <c r="E74" s="16"/>
+      <c r="O74" s="16"/>
+      <c r="P74" s="16"/>
+      <c r="R74" s="16"/>
+      <c r="S74" s="16"/>
+      <c r="T74" s="16"/>
+      <c r="U74" s="16"/>
+      <c r="V74" s="16"/>
+    </row>
+    <row r="75" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A75" s="16"/>
+      <c r="C75" s="16"/>
+      <c r="D75" s="16"/>
+      <c r="E75" s="16"/>
+      <c r="O75" s="16"/>
+      <c r="P75" s="16"/>
+      <c r="R75" s="16"/>
+      <c r="S75" s="16"/>
+      <c r="T75" s="16"/>
+      <c r="U75" s="16"/>
+      <c r="V75" s="16"/>
+    </row>
+    <row r="76" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A76" s="16"/>
+      <c r="C76" s="16"/>
+      <c r="D76" s="16"/>
+      <c r="E76" s="16"/>
+      <c r="O76" s="16"/>
+      <c r="P76" s="16"/>
+      <c r="R76" s="16"/>
+      <c r="S76" s="16"/>
+      <c r="T76" s="16"/>
+      <c r="U76" s="16"/>
+      <c r="V76" s="16"/>
+    </row>
+    <row r="77" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A77" s="16"/>
+      <c r="C77" s="16"/>
+      <c r="D77" s="16"/>
+      <c r="E77" s="16"/>
+      <c r="O77" s="16"/>
+      <c r="P77" s="16"/>
+      <c r="R77" s="16"/>
+      <c r="S77" s="16"/>
+      <c r="T77" s="16"/>
+      <c r="U77" s="16"/>
+      <c r="V77" s="16"/>
+    </row>
+    <row r="78" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A78" s="16"/>
+      <c r="C78" s="16"/>
+      <c r="D78" s="16"/>
+      <c r="E78" s="16"/>
+      <c r="O78" s="16"/>
+      <c r="P78" s="16"/>
+      <c r="R78" s="16"/>
+      <c r="S78" s="16"/>
+      <c r="T78" s="16"/>
+      <c r="U78" s="16"/>
+      <c r="V78" s="16"/>
+    </row>
+    <row r="79" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A79" s="16"/>
+      <c r="C79" s="16"/>
+      <c r="D79" s="16"/>
+      <c r="E79" s="16"/>
+      <c r="O79" s="16"/>
+      <c r="P79" s="16"/>
+      <c r="R79" s="16"/>
+      <c r="S79" s="16"/>
+      <c r="T79" s="16"/>
+      <c r="U79" s="16"/>
+      <c r="V79" s="16"/>
+    </row>
+    <row r="80" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A80" s="16"/>
+      <c r="C80" s="16"/>
+      <c r="D80" s="16"/>
+      <c r="E80" s="16"/>
+      <c r="O80" s="16"/>
+      <c r="P80" s="16"/>
+      <c r="R80" s="16"/>
+      <c r="S80" s="16"/>
+      <c r="T80" s="16"/>
+      <c r="U80" s="16"/>
+      <c r="V80" s="16"/>
+    </row>
+    <row r="81" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A81" s="16"/>
+      <c r="C81" s="16"/>
+      <c r="D81" s="16"/>
+      <c r="E81" s="16"/>
+      <c r="O81" s="16"/>
+      <c r="P81" s="16"/>
+      <c r="R81" s="16"/>
+      <c r="S81" s="16"/>
+      <c r="T81" s="16"/>
+      <c r="U81" s="16"/>
+      <c r="V81" s="16"/>
+    </row>
+    <row r="82" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A82" s="16"/>
+      <c r="C82" s="16"/>
+      <c r="D82" s="16"/>
+      <c r="E82" s="16"/>
+      <c r="O82" s="16"/>
+      <c r="P82" s="16"/>
+      <c r="R82" s="16"/>
+      <c r="S82" s="16"/>
+      <c r="T82" s="16"/>
+      <c r="U82" s="16"/>
+      <c r="V82" s="16"/>
+    </row>
+    <row r="83" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A83" s="16"/>
+      <c r="C83" s="16"/>
+      <c r="D83" s="16"/>
+      <c r="E83" s="16"/>
+      <c r="O83" s="16"/>
+      <c r="P83" s="16"/>
+      <c r="R83" s="16"/>
+      <c r="S83" s="16"/>
+      <c r="T83" s="16"/>
+      <c r="U83" s="16"/>
+      <c r="V83" s="16"/>
+    </row>
+    <row r="84" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A84" s="16"/>
+      <c r="C84" s="16"/>
+      <c r="D84" s="16"/>
+      <c r="E84" s="16"/>
+      <c r="O84" s="16"/>
+      <c r="P84" s="16"/>
+      <c r="R84" s="16"/>
+      <c r="S84" s="16"/>
+      <c r="T84" s="16"/>
+      <c r="U84" s="16"/>
+      <c r="V84" s="16"/>
+    </row>
+    <row r="85" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A85" s="16"/>
+      <c r="C85" s="16"/>
+      <c r="D85" s="16"/>
+      <c r="E85" s="16"/>
+      <c r="O85" s="16"/>
+      <c r="P85" s="16"/>
+      <c r="R85" s="16"/>
+      <c r="S85" s="16"/>
+      <c r="T85" s="16"/>
+      <c r="U85" s="16"/>
+      <c r="V85" s="16"/>
+    </row>
+    <row r="86" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A86" s="16"/>
+      <c r="C86" s="16"/>
+      <c r="D86" s="16"/>
+      <c r="E86" s="16"/>
+      <c r="O86" s="16"/>
+      <c r="P86" s="16"/>
+      <c r="R86" s="16"/>
+      <c r="S86" s="16"/>
+      <c r="T86" s="16"/>
+      <c r="U86" s="16"/>
+      <c r="V86" s="16"/>
+    </row>
+    <row r="87" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A87" s="16"/>
+      <c r="C87" s="16"/>
+      <c r="D87" s="16"/>
+      <c r="E87" s="16"/>
+      <c r="O87" s="16"/>
+      <c r="P87" s="16"/>
+      <c r="R87" s="16"/>
+      <c r="S87" s="16"/>
+      <c r="T87" s="16"/>
+      <c r="U87" s="16"/>
+      <c r="V87" s="16"/>
+    </row>
+    <row r="88" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A88" s="16"/>
+      <c r="C88" s="16"/>
+      <c r="D88" s="16"/>
+      <c r="E88" s="16"/>
+      <c r="O88" s="16"/>
+      <c r="P88" s="16"/>
+      <c r="R88" s="16"/>
+      <c r="S88" s="16"/>
+      <c r="T88" s="16"/>
+      <c r="U88" s="16"/>
+      <c r="V88" s="16"/>
+    </row>
+    <row r="89" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A89" s="16"/>
+      <c r="C89" s="16"/>
+      <c r="D89" s="16"/>
+      <c r="E89" s="16"/>
+      <c r="O89" s="16"/>
+      <c r="P89" s="16"/>
+      <c r="R89" s="16"/>
+      <c r="S89" s="16"/>
+      <c r="T89" s="16"/>
+      <c r="U89" s="16"/>
+      <c r="V89" s="16"/>
+    </row>
+    <row r="90" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A90" s="16"/>
+      <c r="C90" s="16"/>
+      <c r="D90" s="16"/>
+      <c r="E90" s="16"/>
+      <c r="O90" s="16"/>
+      <c r="P90" s="16"/>
+      <c r="R90" s="16"/>
+      <c r="S90" s="16"/>
+      <c r="T90" s="16"/>
+      <c r="U90" s="16"/>
+      <c r="V90" s="16"/>
+    </row>
+    <row r="91" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A91" s="16"/>
+      <c r="C91" s="16"/>
+      <c r="D91" s="16"/>
+      <c r="E91" s="16"/>
+      <c r="O91" s="16"/>
+      <c r="P91" s="16"/>
+      <c r="R91" s="16"/>
+      <c r="S91" s="16"/>
+      <c r="T91" s="16"/>
+      <c r="U91" s="16"/>
+      <c r="V91" s="16"/>
+    </row>
+    <row r="92" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A92" s="16"/>
+      <c r="C92" s="16"/>
+      <c r="D92" s="16"/>
+      <c r="E92" s="16"/>
+      <c r="O92" s="16"/>
+      <c r="P92" s="16"/>
+      <c r="R92" s="16"/>
+      <c r="S92" s="16"/>
+      <c r="T92" s="16"/>
+      <c r="U92" s="16"/>
+      <c r="V92" s="16"/>
+    </row>
+    <row r="93" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A93" s="16"/>
+      <c r="C93" s="16"/>
+      <c r="D93" s="16"/>
+      <c r="E93" s="16"/>
+      <c r="O93" s="16"/>
+      <c r="P93" s="16"/>
+      <c r="R93" s="16"/>
+      <c r="S93" s="16"/>
+      <c r="T93" s="16"/>
+      <c r="U93" s="16"/>
+      <c r="V93" s="16"/>
+    </row>
+    <row r="94" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A94" s="16"/>
+      <c r="C94" s="16"/>
+      <c r="D94" s="16"/>
+      <c r="E94" s="16"/>
+      <c r="O94" s="16"/>
+      <c r="P94" s="16"/>
+      <c r="R94" s="16"/>
+      <c r="S94" s="16"/>
+      <c r="T94" s="16"/>
+      <c r="U94" s="16"/>
+      <c r="V94" s="16"/>
+    </row>
+    <row r="95" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A95" s="16"/>
+      <c r="C95" s="16"/>
+      <c r="D95" s="16"/>
+      <c r="E95" s="16"/>
+      <c r="O95" s="16"/>
+      <c r="P95" s="16"/>
+      <c r="R95" s="16"/>
+      <c r="S95" s="16"/>
+      <c r="T95" s="16"/>
+      <c r="U95" s="16"/>
+      <c r="V95" s="16"/>
+    </row>
+    <row r="96" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A96" s="16"/>
+      <c r="C96" s="16"/>
+      <c r="D96" s="16"/>
+      <c r="E96" s="16"/>
+      <c r="O96" s="16"/>
+      <c r="P96" s="16"/>
+      <c r="R96" s="16"/>
+      <c r="S96" s="16"/>
+      <c r="T96" s="16"/>
+      <c r="U96" s="16"/>
+      <c r="V96" s="16"/>
+    </row>
+    <row r="97" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A97" s="16"/>
+      <c r="C97" s="16"/>
+      <c r="D97" s="16"/>
+      <c r="E97" s="16"/>
+      <c r="O97" s="16"/>
+      <c r="P97" s="16"/>
+      <c r="R97" s="16"/>
+      <c r="S97" s="16"/>
+      <c r="T97" s="16"/>
+      <c r="U97" s="16"/>
+      <c r="V97" s="16"/>
+    </row>
+    <row r="98" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A98" s="16"/>
+      <c r="C98" s="16"/>
+      <c r="D98" s="16"/>
+      <c r="E98" s="16"/>
+      <c r="O98" s="16"/>
+      <c r="P98" s="16"/>
+      <c r="R98" s="16"/>
+      <c r="S98" s="16"/>
+      <c r="T98" s="16"/>
+      <c r="U98" s="16"/>
+      <c r="V98" s="16"/>
+    </row>
+    <row r="99" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A99" s="16"/>
+      <c r="C99" s="16"/>
+      <c r="D99" s="16"/>
+      <c r="E99" s="16"/>
+      <c r="O99" s="16"/>
+      <c r="P99" s="16"/>
+      <c r="R99" s="16"/>
+      <c r="S99" s="16"/>
+      <c r="T99" s="16"/>
+      <c r="U99" s="16"/>
+      <c r="V99" s="16"/>
+    </row>
+    <row r="100" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A100" s="16"/>
+      <c r="C100" s="16"/>
+      <c r="D100" s="16"/>
+      <c r="E100" s="16"/>
+      <c r="O100" s="16"/>
+      <c r="P100" s="16"/>
+      <c r="R100" s="16"/>
+      <c r="S100" s="16"/>
+      <c r="T100" s="16"/>
+      <c r="U100" s="16"/>
+      <c r="V100" s="16"/>
+    </row>
+    <row r="101" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A101" s="16"/>
+      <c r="C101" s="16"/>
+      <c r="D101" s="16"/>
+      <c r="E101" s="16"/>
+      <c r="O101" s="16"/>
+      <c r="P101" s="16"/>
+      <c r="R101" s="16"/>
+      <c r="S101" s="16"/>
+      <c r="T101" s="16"/>
+      <c r="U101" s="16"/>
+      <c r="V101" s="16"/>
+    </row>
+    <row r="102" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A102" s="16"/>
+      <c r="C102" s="16"/>
+      <c r="D102" s="16"/>
+      <c r="E102" s="16"/>
+      <c r="O102" s="16"/>
+      <c r="P102" s="16"/>
+      <c r="R102" s="16"/>
+      <c r="S102" s="16"/>
+      <c r="T102" s="16"/>
+      <c r="U102" s="16"/>
+      <c r="V102" s="16"/>
+    </row>
+    <row r="103" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A103" s="16"/>
+      <c r="C103" s="16"/>
+      <c r="D103" s="16"/>
+      <c r="E103" s="16"/>
+      <c r="O103" s="16"/>
+      <c r="P103" s="16"/>
+      <c r="R103" s="16"/>
+      <c r="S103" s="16"/>
+      <c r="T103" s="16"/>
+      <c r="U103" s="16"/>
+      <c r="V103" s="16"/>
+    </row>
+    <row r="104" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A104" s="16"/>
+      <c r="C104" s="16"/>
+      <c r="D104" s="16"/>
+      <c r="E104" s="16"/>
+      <c r="O104" s="16"/>
+      <c r="P104" s="16"/>
+      <c r="R104" s="16"/>
+      <c r="S104" s="16"/>
+      <c r="T104" s="16"/>
+      <c r="U104" s="16"/>
+      <c r="V104" s="16"/>
+    </row>
+    <row r="105" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A105" s="16"/>
+      <c r="C105" s="16"/>
+      <c r="D105" s="16"/>
+      <c r="E105" s="16"/>
+      <c r="O105" s="16"/>
+      <c r="P105" s="16"/>
+      <c r="R105" s="16"/>
+      <c r="S105" s="16"/>
+      <c r="T105" s="16"/>
+      <c r="U105" s="16"/>
+      <c r="V105" s="16"/>
+    </row>
+    <row r="106" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A106" s="16"/>
+      <c r="C106" s="16"/>
+      <c r="D106" s="16"/>
+      <c r="E106" s="16"/>
+      <c r="O106" s="16"/>
+      <c r="P106" s="16"/>
+      <c r="R106" s="16"/>
+      <c r="S106" s="16"/>
+      <c r="T106" s="16"/>
+      <c r="U106" s="16"/>
+      <c r="V106" s="16"/>
+    </row>
+    <row r="107" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A107" s="16"/>
+      <c r="C107" s="16"/>
+      <c r="D107" s="16"/>
+      <c r="E107" s="16"/>
+      <c r="O107" s="16"/>
+      <c r="P107" s="16"/>
+      <c r="R107" s="16"/>
+      <c r="S107" s="16"/>
+      <c r="T107" s="16"/>
+      <c r="U107" s="16"/>
+      <c r="V107" s="16"/>
+    </row>
+    <row r="108" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A108" s="16"/>
+      <c r="C108" s="16"/>
+      <c r="D108" s="16"/>
+      <c r="E108" s="16"/>
+      <c r="O108" s="16"/>
+      <c r="P108" s="16"/>
+      <c r="R108" s="16"/>
+      <c r="S108" s="16"/>
+      <c r="T108" s="16"/>
+      <c r="U108" s="16"/>
+      <c r="V108" s="16"/>
+    </row>
+    <row r="109" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A109" s="16"/>
+      <c r="C109" s="16"/>
+      <c r="D109" s="16"/>
+      <c r="E109" s="16"/>
+      <c r="O109" s="16"/>
+      <c r="P109" s="16"/>
+      <c r="R109" s="16"/>
+      <c r="S109" s="16"/>
+      <c r="T109" s="16"/>
+      <c r="U109" s="16"/>
+      <c r="V109" s="16"/>
+    </row>
+    <row r="110" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A110" s="16"/>
+      <c r="C110" s="16"/>
+      <c r="D110" s="16"/>
+      <c r="E110" s="16"/>
+      <c r="O110" s="16"/>
+      <c r="P110" s="16"/>
+      <c r="R110" s="16"/>
+      <c r="S110" s="16"/>
+      <c r="T110" s="16"/>
+      <c r="U110" s="16"/>
+      <c r="V110" s="16"/>
+    </row>
+    <row r="111" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A111" s="16"/>
+      <c r="C111" s="16"/>
+      <c r="D111" s="16"/>
+      <c r="E111" s="16"/>
+      <c r="O111" s="16"/>
+      <c r="P111" s="16"/>
+      <c r="R111" s="16"/>
+      <c r="S111" s="16"/>
+      <c r="T111" s="16"/>
+      <c r="U111" s="16"/>
+      <c r="V111" s="16"/>
+    </row>
+    <row r="112" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A112" s="16"/>
+      <c r="C112" s="16"/>
+      <c r="D112" s="16"/>
+      <c r="E112" s="16"/>
+      <c r="O112" s="16"/>
+      <c r="P112" s="16"/>
+      <c r="R112" s="16"/>
+      <c r="S112" s="16"/>
+      <c r="T112" s="16"/>
+      <c r="U112" s="16"/>
+      <c r="V112" s="16"/>
+    </row>
+    <row r="113" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A113" s="16"/>
+      <c r="C113" s="16"/>
+      <c r="D113" s="16"/>
+      <c r="E113" s="16"/>
+      <c r="O113" s="16"/>
+      <c r="P113" s="16"/>
+      <c r="R113" s="16"/>
+      <c r="S113" s="16"/>
+      <c r="T113" s="16"/>
+      <c r="U113" s="16"/>
+      <c r="V113" s="16"/>
+    </row>
+    <row r="114" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A114" s="16"/>
+      <c r="C114" s="16"/>
+      <c r="D114" s="16"/>
+      <c r="E114" s="16"/>
+      <c r="O114" s="16"/>
+      <c r="P114" s="16"/>
+      <c r="R114" s="16"/>
+      <c r="S114" s="16"/>
+      <c r="T114" s="16"/>
+      <c r="U114" s="16"/>
+      <c r="V114" s="16"/>
+    </row>
+    <row r="115" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A115" s="16"/>
+      <c r="C115" s="16"/>
+      <c r="D115" s="16"/>
+      <c r="E115" s="16"/>
+      <c r="O115" s="16"/>
+      <c r="P115" s="16"/>
+      <c r="R115" s="16"/>
+      <c r="S115" s="16"/>
+      <c r="T115" s="16"/>
+      <c r="U115" s="16"/>
+      <c r="V115" s="16"/>
+    </row>
+    <row r="116" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A116" s="16"/>
+      <c r="C116" s="16"/>
+      <c r="D116" s="16"/>
+      <c r="E116" s="16"/>
+      <c r="O116" s="16"/>
+      <c r="P116" s="16"/>
+      <c r="R116" s="16"/>
+      <c r="S116" s="16"/>
+      <c r="T116" s="16"/>
+      <c r="U116" s="16"/>
+      <c r="V116" s="16"/>
+    </row>
+    <row r="117" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A117" s="16"/>
+      <c r="C117" s="16"/>
+      <c r="D117" s="16"/>
+      <c r="E117" s="16"/>
+      <c r="O117" s="16"/>
+      <c r="P117" s="16"/>
+      <c r="R117" s="16"/>
+      <c r="S117" s="16"/>
+      <c r="T117" s="16"/>
+      <c r="U117" s="16"/>
+      <c r="V117" s="16"/>
+    </row>
+    <row r="118" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A118" s="16"/>
+      <c r="C118" s="16"/>
+      <c r="D118" s="16"/>
+      <c r="E118" s="16"/>
+      <c r="O118" s="16"/>
+      <c r="P118" s="16"/>
+      <c r="R118" s="16"/>
+      <c r="S118" s="16"/>
+      <c r="T118" s="16"/>
+      <c r="U118" s="16"/>
+      <c r="V118" s="16"/>
+    </row>
+    <row r="119" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A119" s="16"/>
+      <c r="C119" s="16"/>
+      <c r="D119" s="16"/>
+      <c r="E119" s="16"/>
+      <c r="O119" s="16"/>
+      <c r="P119" s="16"/>
+      <c r="R119" s="16"/>
+      <c r="S119" s="16"/>
+      <c r="T119" s="16"/>
+      <c r="U119" s="16"/>
+      <c r="V119" s="16"/>
+    </row>
+    <row r="120" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A120" s="16"/>
+      <c r="C120" s="16"/>
+      <c r="D120" s="16"/>
+      <c r="E120" s="16"/>
+      <c r="O120" s="16"/>
+      <c r="P120" s="16"/>
+      <c r="R120" s="16"/>
+      <c r="S120" s="16"/>
+      <c r="T120" s="16"/>
+      <c r="U120" s="16"/>
+      <c r="V120" s="16"/>
+    </row>
+    <row r="121" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A121" s="16"/>
+      <c r="C121" s="16"/>
+      <c r="D121" s="16"/>
+      <c r="E121" s="16"/>
+      <c r="O121" s="16"/>
+      <c r="P121" s="16"/>
+      <c r="R121" s="16"/>
+      <c r="S121" s="16"/>
+      <c r="T121" s="16"/>
+      <c r="U121" s="16"/>
+      <c r="V121" s="16"/>
+    </row>
+    <row r="122" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A122" s="16"/>
+      <c r="C122" s="16"/>
+      <c r="D122" s="16"/>
+      <c r="E122" s="16"/>
+      <c r="O122" s="16"/>
+      <c r="P122" s="16"/>
+      <c r="R122" s="16"/>
+      <c r="S122" s="16"/>
+      <c r="T122" s="16"/>
+      <c r="U122" s="16"/>
+      <c r="V122" s="16"/>
+    </row>
+    <row r="123" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A123" s="16"/>
+      <c r="C123" s="16"/>
+      <c r="D123" s="16"/>
+      <c r="E123" s="16"/>
+      <c r="O123" s="16"/>
+      <c r="P123" s="16"/>
+      <c r="R123" s="16"/>
+      <c r="S123" s="16"/>
+      <c r="T123" s="16"/>
+      <c r="U123" s="16"/>
+      <c r="V123" s="16"/>
+    </row>
+    <row r="124" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A124" s="16"/>
+      <c r="C124" s="16"/>
+      <c r="D124" s="16"/>
+      <c r="E124" s="16"/>
+      <c r="O124" s="16"/>
+      <c r="P124" s="16"/>
+      <c r="R124" s="16"/>
+      <c r="S124" s="16"/>
+      <c r="T124" s="16"/>
+      <c r="U124" s="16"/>
+      <c r="V124" s="16"/>
+    </row>
+    <row r="125" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A125" s="16"/>
+      <c r="C125" s="16"/>
+      <c r="D125" s="16"/>
+      <c r="E125" s="16"/>
+      <c r="O125" s="16"/>
+      <c r="P125" s="16"/>
+      <c r="R125" s="16"/>
+      <c r="S125" s="16"/>
+      <c r="T125" s="16"/>
+      <c r="U125" s="16"/>
+      <c r="V125" s="16"/>
+    </row>
+    <row r="126" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A126" s="16"/>
+      <c r="C126" s="16"/>
+      <c r="D126" s="16"/>
+      <c r="E126" s="16"/>
+      <c r="O126" s="16"/>
+      <c r="P126" s="16"/>
+      <c r="R126" s="16"/>
+      <c r="S126" s="16"/>
+      <c r="T126" s="16"/>
+      <c r="U126" s="16"/>
+      <c r="V126" s="16"/>
+    </row>
+    <row r="127" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A127" s="16"/>
+      <c r="C127" s="16"/>
+      <c r="D127" s="16"/>
+      <c r="E127" s="16"/>
+      <c r="O127" s="16"/>
+      <c r="P127" s="16"/>
+      <c r="R127" s="16"/>
+      <c r="S127" s="16"/>
+      <c r="T127" s="16"/>
+      <c r="U127" s="16"/>
+      <c r="V127" s="16"/>
+    </row>
+    <row r="128" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A128" s="16"/>
+      <c r="C128" s="16"/>
+      <c r="D128" s="16"/>
+      <c r="E128" s="16"/>
+      <c r="O128" s="16"/>
+      <c r="P128" s="16"/>
+      <c r="R128" s="16"/>
+      <c r="S128" s="16"/>
+      <c r="T128" s="16"/>
+      <c r="U128" s="16"/>
+      <c r="V128" s="16"/>
+    </row>
+    <row r="129" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A129" s="16"/>
+      <c r="C129" s="16"/>
+      <c r="D129" s="16"/>
+      <c r="E129" s="16"/>
+      <c r="O129" s="16"/>
+      <c r="P129" s="16"/>
+      <c r="R129" s="16"/>
+      <c r="S129" s="16"/>
+      <c r="T129" s="16"/>
+      <c r="U129" s="16"/>
+      <c r="V129" s="16"/>
+    </row>
+    <row r="130" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A130" s="16"/>
+      <c r="C130" s="16"/>
+      <c r="D130" s="16"/>
+      <c r="E130" s="16"/>
+      <c r="O130" s="16"/>
+      <c r="P130" s="16"/>
+      <c r="R130" s="16"/>
+      <c r="S130" s="16"/>
+      <c r="T130" s="16"/>
+      <c r="U130" s="16"/>
+      <c r="V130" s="16"/>
+    </row>
+    <row r="131" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A131" s="16"/>
+      <c r="C131" s="16"/>
+      <c r="D131" s="16"/>
+      <c r="E131" s="16"/>
+      <c r="O131" s="16"/>
+      <c r="P131" s="16"/>
+      <c r="R131" s="16"/>
+      <c r="S131" s="16"/>
+      <c r="T131" s="16"/>
+      <c r="U131" s="16"/>
+      <c r="V131" s="16"/>
+    </row>
+    <row r="132" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A132" s="16"/>
+      <c r="C132" s="16"/>
+      <c r="D132" s="16"/>
+      <c r="E132" s="16"/>
+      <c r="O132" s="16"/>
+      <c r="P132" s="16"/>
+      <c r="R132" s="16"/>
+      <c r="S132" s="16"/>
+      <c r="T132" s="16"/>
+      <c r="U132" s="16"/>
+      <c r="V132" s="16"/>
+    </row>
+    <row r="133" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A133" s="16"/>
+      <c r="C133" s="16"/>
+      <c r="D133" s="16"/>
+      <c r="E133" s="16"/>
+      <c r="O133" s="16"/>
+      <c r="P133" s="16"/>
+      <c r="R133" s="16"/>
+      <c r="S133" s="16"/>
+      <c r="T133" s="16"/>
+      <c r="U133" s="16"/>
+      <c r="V133" s="16"/>
+    </row>
+    <row r="134" spans="1:22" x14ac:dyDescent="0.5">
+      <c r="A134" s="16"/>
+      <c r="C134" s="16"/>
+      <c r="D134" s="16"/>
+      <c r="E134" s="16"/>
+      <c r="O134" s="16"/>
+      <c r="P134" s="16"/>
+      <c r="R134" s="16"/>
+      <c r="S134" s="16"/>
+      <c r="T134" s="16"/>
+      <c r="U134" s="16"/>
+      <c r="V134" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="B2:E2"/>
   </mergeCells>
+  <phoneticPr fontId="13" type="noConversion"/>
   <dataValidations count="6">
-    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Количество символов не должно превышать 90 знаков" sqref="E5:E6 E37:E1048576 I5:I1048576 M5:M1048576">
-      <formula1>91</formula1>
+    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Количество символов не должно превышать 70 знаков" sqref="A5:B21 A135:A1048576 B122:B123 B113:B115 B26:B27 B22:B23 B30:B32 B34:B38 B62:B64 B41:B42 B45:B46 B49:B51 B58:B59 B54:B55 B130:B1048576 B66:B70 B86:B87 B94:B96 B73:B74 B77:B78 B81:B83 B90:B91 B98:B102 B118:B119 B126:B128 B105:B106 B109:B110">
+      <formula1>71</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L5:L6 H5:H6 H26:H1048576 L15:L21 L26:L1048576 H15:H21">
+    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Количество символов не должно превышать 90 знаков" sqref="E5:E6 E135:E1048576 I5:I1048576 M5:M1048576">
       <formula1>91</formula1>
     </dataValidation>
     <dataValidation operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H4 L3:L4"/>
-    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Количество символов не должно превышать 35 знаков" sqref="L22:L25 H22:H25 L7:L14 H7:H14">
+    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Количество символов не должно превышать 35 знаков" sqref="D135:D1048576 D5:D102">
+      <formula1>91</formula1>
+    </dataValidation>
+    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H22:H1048576 H5:H6 L5:L6 L22:L1048576">
+      <formula1>91</formula1>
+    </dataValidation>
+    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Количество символов не должно превышать 35 знаков" sqref="H7:H21 L7:L21">
       <formula1>36</formula1>
-    </dataValidation>
-    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Количество символов не должно превышать 70 знаков" sqref="A26:A1048576 B28:B1048576 A5:B25">
-      <formula1>71</formula1>
-    </dataValidation>
-    <dataValidation type="textLength" operator="lessThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Количество символов не должно превышать 35 знаков" sqref="D5:D1048576">
-      <formula1>91</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="203" r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>catalogues!$A$2:$A$185</xm:f>
           </x14:formula1>
-          <xm:sqref>G37:G1048576 C37:C1048576 K6 G6 C6 K37:K1048576</xm:sqref>
+          <xm:sqref>C6 C135:C1048576 G22:G1048576 G6 K6 K22:K1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>catalogues!$B$2:$B$253</xm:f>
           </x14:formula1>
-          <xm:sqref>O6:Q6 O37:Q1048576</xm:sqref>
+          <xm:sqref>O6:Q6 O135:P1048576 Q22:Q1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>catalogues!$C$2:$C$41</xm:f>
           </x14:formula1>
-          <xm:sqref>T6 T37:T1048576</xm:sqref>
+          <xm:sqref>T6 T135:T1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>catalogues!$E$2:$E$3</xm:f>
           </x14:formula1>
-          <xm:sqref>V6 V37:V1048576</xm:sqref>
+          <xm:sqref>V6 V135:V1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>catalogues!$D$2:$D$3</xm:f>
           </x14:formula1>
-          <xm:sqref>U6 U37:U1048576</xm:sqref>
+          <xm:sqref>U6 U135:U1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>[1]catalogues!#REF!</xm:f>
+          </x14:formula1>
+          <xm:sqref>T22:V134 C22:C134 O22:P134</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3406,7 +5117,7 @@
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="25.86328125" customWidth="1"/>
     <col min="3" max="3" width="35.86328125" customWidth="1"/>
-    <col min="4" max="4" width="33.3984375" customWidth="1"/>
+    <col min="4" max="4" width="33.46484375" customWidth="1"/>
     <col min="5" max="5" width="31.86328125" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>